<commit_message>
Freigaben dauerhaft einstellen, Nr. 155 entschieden
- .claude/settings.json: Webflow-, Datei-, Shell- und Web-Werkzeuge ohne
  Rueckfrage erlaubt; Force-Push und Hard-Reset gesperrt
- Redirect-Mapping: Nr. 155 entfaellt, Nr. 156 wieder 301 auf
  /persoenliche-entwicklung; alle 166 Zeilen entschieden
- Report 7.1 (E4) nachgefuehrt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WRYKhSHh6BQB8xQaR7BU5Z
</commit_message>
<xml_diff>
--- a/exports/02_redirect_mapping.xlsx
+++ b/exports/02_redirect_mapping.xlsx
@@ -1175,13 +1175,13 @@
     <t xml:space="preserve">https://rowapa.ch/training-kategorie/exklusiv/</t>
   </si>
   <si>
-    <t xml:space="preserve">Vorschlag – prüfen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">„Exklusiv“ hat keine Entsprechung → Übersicht.</t>
+    <t xml:space="preserve">Entscheid ROWAPA 25.10.2026: Kategorie «Exklusiv» gibt es nicht mehr, Seite entfällt.</t>
   </si>
   <si>
     <t xml:space="preserve">https://rowapa.ch/training-kategorie/kurse/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shop-Kategorie Kurse → Übersicht persönliche Entwicklung.</t>
   </si>
   <si>
     <t xml:space="preserve">https://rowapa.ch/training-kategorie/leadership/</t>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="F9" s="7" t="n">
         <f aca="false">COUNTIF('Alt-URLs (rowapa.ch)'!$H$2:$H$167,"sicher")</f>
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="F10" s="7" t="n">
         <f aca="false">COUNTIF('Alt-URLs (rowapa.ch)'!$H$2:$H$167,"Vorschlag – prüfen")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6404,17 +6404,17 @@
         <v>22</v>
       </c>
       <c r="E156" s="15" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F156" s="15" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G156" s="17"/>
       <c r="H156" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="I156" s="17" t="s">
         <v>383</v>
-      </c>
-      <c r="I156" s="17" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6422,7 +6422,7 @@
         <v>156</v>
       </c>
       <c r="B157" s="19" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C157" s="19" t="s">
         <v>24</v>
@@ -6431,17 +6431,17 @@
         <v>22</v>
       </c>
       <c r="E157" s="19" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F157" s="19" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G157" s="20"/>
       <c r="H157" s="20" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="I157" s="20" t="s">
-        <v>60</v>
+        <v>385</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>